<commit_message>
FEAT/FIX: errores corregidos y funcionalidades añadidas (paso2 y prog obj)
Se hacen correctamente los ensamblados con sus respectivos manejos de errores, se solucionaron bugs
</commit_message>
<xml_diff>
--- a/ProyectoSoftwareSistemas/bin/Debug/output/PRINCIPAL_CLASE_ArchivoIntermedio.xlsx
+++ b/ProyectoSoftwareSistemas/bin/Debug/output/PRINCIPAL_CLASE_ArchivoIntermedio.xlsx
@@ -7,11 +7,12 @@
   </x:bookViews>
   <x:sheets>
     <x:sheet name="ArchivoIntermedio" sheetId="1" r:id="rId2"/>
-    <x:sheet name="ProgramaObjeto" sheetId="2" r:id="rId3"/>
-    <x:sheet name="TABBLK_DEFAULT" sheetId="3" r:id="rId4"/>
+    <x:sheet name="ProgObj_PRINCI" sheetId="2" r:id="rId3"/>
+    <x:sheet name="ProgObj_MODULO" sheetId="3" r:id="rId4"/>
     <x:sheet name="TABSIM_DEFAULT" sheetId="4" r:id="rId5"/>
-    <x:sheet name="TABBLK_MODULO" sheetId="5" r:id="rId6"/>
+    <x:sheet name="TABBLK_DEFAULT" sheetId="5" r:id="rId6"/>
     <x:sheet name="TABSIM_MODULO" sheetId="6" r:id="rId7"/>
+    <x:sheet name="TABBLK_MODULO" sheetId="7" r:id="rId8"/>
   </x:sheets>
   <x:definedNames/>
   <x:calcPr calcId="125725"/>
@@ -171,10 +172,7 @@
     <x:t>RETADR</x:t>
   </x:si>
   <x:si>
-    <x:t>Símbolo no definido: RETADR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>176FFF</x:t>
+    <x:t>172012</x:t>
   </x:si>
   <x:si>
     <x:t>0003</x:t>
@@ -207,10 +205,7 @@
     <x:t>RDREC</x:t>
   </x:si>
   <x:si>
-    <x:t>Símbolo no definido: RDREC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>4B6FFF</x:t>
+    <x:t>4B2003</x:t>
   </x:si>
   <x:si>
     <x:t>0008</x:t>
@@ -219,10 +214,7 @@
     <x:t>LENGTH</x:t>
   </x:si>
   <x:si>
-    <x:t>Símbolo no definido: LENGTH</x:t>
-  </x:si>
-  <x:si>
-    <x:t>036FFF</x:t>
+    <x:t>032010</x:t>
   </x:si>
   <x:si>
     <x:t>USE</x:t>
@@ -255,7 +247,7 @@
     <x:t>ENDA+6</x:t>
   </x:si>
   <x:si>
-    <x:t>000010*R</x:t>
+    <x:t>000006*SE</x:t>
   </x:si>
   <x:si>
     <x:t>1003</x:t>
@@ -270,16 +262,10 @@
     <x:t>BUFFEND-BUFFER+3</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Error: Símbolos de diferentes bloques en EQU | </x:t>
-  </x:si>
-  <x:si>
     <x:t>BUFFEND+6</x:t>
   </x:si>
   <x:si>
-    <x:t>Símbolo no definido: BUFFEND</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FFFFFF</x:t>
+    <x:t>00102F*R</x:t>
   </x:si>
   <x:si>
     <x:t>000B</x:t>
@@ -300,10 +286,7 @@
     <x:t>#MAXLEN</x:t>
   </x:si>
   <x:si>
-    <x:t>Símbolo no definido: MAXLEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>753FFFFF</x:t>
+    <x:t>75101006</x:t>
   </x:si>
   <x:si>
     <x:t>000F</x:t>
@@ -324,33 +307,114 @@
     <x:t>0011</x:t>
   </x:si>
   <x:si>
-    <x:t>7710000A*R</x:t>
+    <x:t>77100000*SE</x:t>
   </x:si>
   <x:si>
     <x:t>END</x:t>
   </x:si>
   <x:si>
+    <x:t>Símbolo no definido: REF2</x:t>
+  </x:si>
+  <x:si>
     <x:t>HPRINCI00000000000A</x:t>
   </x:si>
   <x:si>
-    <x:t>T0000001A03100006*SE01000800000E*R*SE*SE176FFFB4004B6FFF036FFF</x:t>
-  </x:si>
-  <x:si>
-    <x:t>T00100007000010*RFFFFFF</x:t>
-  </x:si>
-  <x:si>
-    <x:t>T00000B06B410753FFFFF</x:t>
-  </x:si>
-  <x:si>
-    <x:t>T00000F0200F1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>T000011057710000A*R</x:t>
+    <x:t>DLISTA 000007</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">RLISTB ENDB  </x:t>
+  </x:si>
+  <x:si>
+    <x:t>DENDA  00000A</x:t>
+  </x:si>
+  <x:si>
+    <x:t>T0000000A0310000601000800000E</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">M00000105+LISTB </x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">M00000706-ENDB  </x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">M00000706+LISTB </x:t>
+  </x:si>
+  <x:si>
+    <x:t>M00000706+PRINCI</x:t>
   </x:si>
   <x:si>
     <x:t>E000004</x:t>
   </x:si>
   <x:si>
+    <x:t>HMODULO00000000102C</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DBUFFER000026INPUT 000024</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">RENDA  </x:t>
+  </x:si>
+  <x:si>
+    <x:t>T0000000B172012B4004B2003032010</x:t>
+  </x:si>
+  <x:si>
+    <x:t>T0010260600000600102F</x:t>
+  </x:si>
+  <x:si>
+    <x:t>T00000B06B41075101006</x:t>
+  </x:si>
+  <x:si>
+    <x:t>T0000240200F1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>T0000110477100000</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">M00102606+ENDA  </x:t>
+  </x:si>
+  <x:si>
+    <x:t>M00102906+MODULO</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">M00001205+ENDA  </x:t>
+  </x:si>
+  <x:si>
+    <x:t>E</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Simbolo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Direccion</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Tipo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NumBloq</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SimboloExterno</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LISTB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sí</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENDB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>R</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DEFAULT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>No</x:t>
+  </x:si>
+  <x:si>
     <x:t>No. Bloque</x:t>
   </x:si>
   <x:si>
@@ -363,52 +427,13 @@
     <x:t>Dir Inicial</x:t>
   </x:si>
   <x:si>
-    <x:t>DEFAULT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Simbolo</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Direccion</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Tipo</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NumBloq</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SimboloExterno</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LISTB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>E</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Sí</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENDB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>R</x:t>
-  </x:si>
-  <x:si>
-    <x:t>No</x:t>
+    <x:t>1006</x:t>
   </x:si>
   <x:si>
     <x:t>0015</x:t>
   </x:si>
   <x:si>
-    <x:t>1006</x:t>
-  </x:si>
-  <x:si>
     <x:t>0026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FFFF</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -770,7 +795,7 @@
     <x:col min="6" max="6" width="20.139196" style="0" customWidth="1"/>
     <x:col min="7" max="7" width="9.710625" style="0" customWidth="1"/>
     <x:col min="8" max="8" width="10.139196" style="0" customWidth="1"/>
-    <x:col min="9" max="9" width="43.853482" style="0" customWidth="1"/>
+    <x:col min="9" max="9" width="24.424911" style="0" customWidth="1"/>
     <x:col min="10" max="10" width="15.710625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -1096,7 +1121,7 @@
     </x:row>
     <x:row r="11" spans="1:10">
       <x:c r="A11" s="0">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B11" s="0">
         <x:v>0</x:v>
@@ -1128,7 +1153,7 @@
     </x:row>
     <x:row r="12" spans="1:10">
       <x:c r="A12" s="0">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B12" s="0">
         <x:v>0</x:v>
@@ -1160,7 +1185,7 @@
     </x:row>
     <x:row r="13" spans="1:10">
       <x:c r="A13" s="0">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B13" s="0">
         <x:v>0</x:v>
@@ -1192,7 +1217,7 @@
     </x:row>
     <x:row r="14" spans="1:10">
       <x:c r="A14" s="0">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B14" s="0">
         <x:v>0</x:v>
@@ -1216,62 +1241,62 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="I14" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="J14" s="0" t="s">
         <x:v>50</x:v>
-      </x:c>
-      <x:c r="J14" s="0" t="s">
-        <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:10">
       <x:c r="A15" s="0">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B15" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C15" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="D15" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="E15" s="0" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="D15" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="E15" s="0" t="s">
+      <x:c r="F15" s="0" t="s">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="F15" s="0" t="s">
+      <x:c r="G15" s="0" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="G15" s="0" t="s">
+      <x:c r="H15" s="0" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="H15" s="0" t="s">
+      <x:c r="I15" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="J15" s="0" t="s">
         <x:v>56</x:v>
-      </x:c>
-      <x:c r="I15" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="J15" s="0" t="s">
-        <x:v>57</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:10">
       <x:c r="A16" s="0">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B16" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C16" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="D16" s="0" t="s">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="D16" s="0" t="s">
+      <x:c r="E16" s="0" t="s">
         <x:v>59</x:v>
       </x:c>
-      <x:c r="E16" s="0" t="s">
+      <x:c r="F16" s="0" t="s">
         <x:v>60</x:v>
-      </x:c>
-      <x:c r="F16" s="0" t="s">
-        <x:v>61</x:v>
       </x:c>
       <x:c r="G16" s="0" t="s">
         <x:v>33</x:v>
@@ -1280,21 +1305,21 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="I16" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="J16" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:10">
       <x:c r="A17" s="0">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B17" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C17" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="D17" s="0" t="s">
         <x:v>16</x:v>
@@ -1303,7 +1328,7 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="F17" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="G17" s="0" t="s">
         <x:v>33</x:v>
@@ -1312,15 +1337,15 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="I17" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="J17" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>64</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:10">
       <x:c r="A18" s="0">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B18" s="0">
         <x:v>1</x:v>
@@ -1332,10 +1357,10 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="E18" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="F18" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="G18" s="0" t="s">
         <x:v>14</x:v>
@@ -1352,7 +1377,7 @@
     </x:row>
     <x:row r="19" spans="1:10">
       <x:c r="A19" s="0">
-        <x:v>19</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B19" s="0">
         <x:v>1</x:v>
@@ -1364,10 +1389,10 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="E19" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="F19" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="G19" s="0" t="s">
         <x:v>14</x:v>
@@ -1384,19 +1409,19 @@
     </x:row>
     <x:row r="20" spans="1:10">
       <x:c r="A20" s="0">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="B20" s="0">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C20" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="D20" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="E20" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="F20" s="0" t="s">
         <x:v>33</x:v>
@@ -1416,7 +1441,7 @@
     </x:row>
     <x:row r="21" spans="1:10">
       <x:c r="A21" s="0">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B21" s="0">
         <x:v>2</x:v>
@@ -1428,10 +1453,10 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="E21" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="F21" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="G21" s="0" t="s">
         <x:v>14</x:v>
@@ -1448,7 +1473,7 @@
     </x:row>
     <x:row r="22" spans="1:10">
       <x:c r="A22" s="0">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B22" s="0">
         <x:v>2</x:v>
@@ -1457,13 +1482,13 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="D22" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E22" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F22" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="G22" s="0" t="s">
         <x:v>14</x:v>
@@ -1480,13 +1505,13 @@
     </x:row>
     <x:row r="23" spans="1:10">
       <x:c r="A23" s="0">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B23" s="0">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C23" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="D23" s="0" t="s">
         <x:v>16</x:v>
@@ -1495,7 +1520,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="F23" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="G23" s="0" t="s">
         <x:v>14</x:v>
@@ -1507,21 +1532,21 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="J23" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:10">
       <x:c r="A24" s="0">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B24" s="0">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C24" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D24" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="E24" s="0" t="s">
         <x:v>37</x:v>
@@ -1544,22 +1569,22 @@
     </x:row>
     <x:row r="25" spans="1:10">
       <x:c r="A25" s="0">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="B25" s="0">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C25" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D25" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E25" s="0" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="F25" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="G25" s="0" t="s">
         <x:v>14</x:v>
@@ -1568,7 +1593,7 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="I25" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="J25" s="0" t="s">
         <x:v>17</x:v>
@@ -1576,13 +1601,13 @@
     </x:row>
     <x:row r="26" spans="1:10">
       <x:c r="A26" s="0">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B26" s="0">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C26" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D26" s="0" t="s">
         <x:v>16</x:v>
@@ -1591,7 +1616,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="F26" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="G26" s="0" t="s">
         <x:v>14</x:v>
@@ -1600,27 +1625,27 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="I26" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="J26" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:10">
       <x:c r="A27" s="0">
-        <x:v>27</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B27" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C27" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="D27" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
       <x:c r="E27" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="F27" s="0" t="s">
         <x:v>16</x:v>
@@ -1640,54 +1665,54 @@
     </x:row>
     <x:row r="28" spans="1:10">
       <x:c r="A28" s="0">
-        <x:v>28</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="B28" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C28" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="D28" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E28" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="F28" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="G28" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="H28" s="0" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="H28" s="0" t="s">
-        <x:v>56</x:v>
-      </x:c>
       <x:c r="I28" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
       <x:c r="J28" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:10">
       <x:c r="A29" s="0">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B29" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C29" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D29" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
       <x:c r="E29" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="F29" s="0" t="s">
-        <x:v>92</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="G29" s="0" t="s">
         <x:v>26</x:v>
@@ -1696,30 +1721,30 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="I29" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="J29" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:10">
       <x:c r="A30" s="0">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B30" s="0">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C30" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="D30" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
       <x:c r="E30" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="F30" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="G30" s="0" t="s">
         <x:v>14</x:v>
@@ -1736,22 +1761,22 @@
     </x:row>
     <x:row r="31" spans="1:10">
       <x:c r="A31" s="0">
-        <x:v>31</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B31" s="0">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C31" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="D31" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E31" s="0" t="s">
-        <x:v>97</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="F31" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="G31" s="0" t="s">
         <x:v>14</x:v>
@@ -1763,24 +1788,24 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="J31" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:10">
       <x:c r="A32" s="0">
-        <x:v>32</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="B32" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C32" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="D32" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
       <x:c r="E32" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="F32" s="0" t="s">
         <x:v>16</x:v>
@@ -1800,19 +1825,19 @@
     </x:row>
     <x:row r="33" spans="1:10">
       <x:c r="A33" s="0">
-        <x:v>33</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B33" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C33" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="D33" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
       <x:c r="E33" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="F33" s="0" t="s">
         <x:v>22</x:v>
@@ -1827,12 +1852,12 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="J33" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:10">
       <x:c r="A34" s="0">
-        <x:v>34</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B34" s="0">
         <x:v>0</x:v>
@@ -1844,7 +1869,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="E34" s="0" t="s">
-        <x:v>102</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="F34" s="0" t="s">
         <x:v>30</x:v>
@@ -1856,7 +1881,7 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="I34" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="J34" s="0" t="s">
         <x:v>17</x:v>
@@ -1876,45 +1901,60 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:A7"/>
+  <x:dimension ref="A1:A10"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="66.996339" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="31.567768" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:1">
       <x:c r="A1" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>98</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:1">
       <x:c r="A2" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>99</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:1">
       <x:c r="A3" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>100</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:1">
       <x:c r="A4" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>101</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:1">
       <x:c r="A5" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:1">
       <x:c r="A6" s="0" t="s">
-        <x:v>108</x:v>
+        <x:v>103</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:1">
       <x:c r="A7" s="0" t="s">
-        <x:v>109</x:v>
+        <x:v>104</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:1">
+      <x:c r="A8" s="0" t="s">
+        <x:v>105</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:1">
+      <x:c r="A9" s="0" t="s">
+        <x:v>106</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:1">
+      <x:c r="A10" s="0" t="s">
+        <x:v>107</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1931,40 +1971,70 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:D2"/>
+  <x:dimension ref="A1:A12"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="10.710625" style="0" customWidth="1"/>
-    <x:col min="2" max="3" width="8.853482" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="8.996339" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="34.139196" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:4">
+    <x:row r="1" spans="1:1">
       <x:c r="A1" s="0" t="s">
+        <x:v>108</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:1">
+      <x:c r="A2" s="0" t="s">
+        <x:v>109</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:1">
+      <x:c r="A3" s="0" t="s">
         <x:v>110</x:v>
       </x:c>
-      <x:c r="B1" s="0" t="s">
+    </x:row>
+    <x:row r="4" spans="1:1">
+      <x:c r="A4" s="0" t="s">
         <x:v>111</x:v>
       </x:c>
-      <x:c r="C1" s="0" t="s">
+    </x:row>
+    <x:row r="5" spans="1:1">
+      <x:c r="A5" s="0" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="D1" s="0" t="s">
+    </x:row>
+    <x:row r="6" spans="1:1">
+      <x:c r="A6" s="0" t="s">
         <x:v>113</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" spans="1:4">
-      <x:c r="A2" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B2" s="0" t="s">
+    <x:row r="7" spans="1:1">
+      <x:c r="A7" s="0" t="s">
         <x:v>114</x:v>
       </x:c>
-      <x:c r="C2" s="0" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="D2" s="0" t="s">
-        <x:v>10</x:v>
+    </x:row>
+    <x:row r="8" spans="1:1">
+      <x:c r="A8" s="0" t="s">
+        <x:v>115</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:1">
+      <x:c r="A9" s="0" t="s">
+        <x:v>116</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:1">
+      <x:c r="A10" s="0" t="s">
+        <x:v>117</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:1">
+      <x:c r="A11" s="0" t="s">
+        <x:v>118</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:1">
+      <x:c r="A12" s="0" t="s">
+        <x:v>119</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1993,53 +2063,53 @@
   <x:sheetData>
     <x:row r="1" spans="1:5">
       <x:c r="A1" s="0" t="s">
-        <x:v>115</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>116</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>117</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>118</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>119</x:v>
+        <x:v>124</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:5">
       <x:c r="A2" s="0" t="s">
-        <x:v>120</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>121</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>122</x:v>
+        <x:v>126</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:5">
       <x:c r="A3" s="0" t="s">
-        <x:v>123</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>121</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>122</x:v>
+        <x:v>126</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:5">
@@ -2050,13 +2120,13 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>124</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>125</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:5">
@@ -2067,13 +2137,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>124</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>125</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:5">
@@ -2084,13 +2154,13 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>124</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>125</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:5">
@@ -2101,13 +2171,13 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>124</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>125</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:5">
@@ -2118,13 +2188,13 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>124</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="E8" s="0" t="s">
-        <x:v>125</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2141,7 +2211,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:D4"/>
+  <x:dimension ref="A1:D2"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="10.710625" style="0" customWidth="1"/>
@@ -2151,16 +2221,16 @@
   <x:sheetData>
     <x:row r="1" spans="1:4">
       <x:c r="A1" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>112</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>113</x:v>
+        <x:v>134</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:4">
@@ -2168,41 +2238,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>126</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
         <x:v>10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:4">
-      <x:c r="A3" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>69</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="D3" s="0" t="s">
-        <x:v>126</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:4">
-      <x:c r="A4" s="0">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
-        <x:v>127</x:v>
-      </x:c>
-      <x:c r="D4" s="0" t="s">
-        <x:v>128</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2231,19 +2273,19 @@
   <x:sheetData>
     <x:row r="1" spans="1:5">
       <x:c r="A1" s="0" t="s">
-        <x:v>115</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>116</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>117</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>118</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>119</x:v>
+        <x:v>124</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:5">
@@ -2254,13 +2296,13 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>121</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>122</x:v>
+        <x:v>126</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:5">
@@ -2271,30 +2313,30 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>124</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>125</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:5">
       <x:c r="A4" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>124</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>125</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:5">
@@ -2305,115 +2347,193 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>124</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>125</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:5">
       <x:c r="A6" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>124</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>125</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:5">
       <x:c r="A7" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>124</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>125</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:5">
       <x:c r="A8" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>124</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="E8" s="0" t="s">
-        <x:v>125</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:5">
       <x:c r="A9" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
-        <x:v>129</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="E9" s="0" t="s">
-        <x:v>125</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:5">
       <x:c r="A10" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
-        <x:v>124</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D10" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="E10" s="0" t="s">
-        <x:v>125</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:5">
       <x:c r="A11" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="C11" s="0" t="s">
-        <x:v>124</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D11" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="E11" s="0" t="s">
+        <x:v>130</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:D4"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="10.710625" style="0" customWidth="1"/>
+    <x:col min="2" max="3" width="8.853482" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8.996339" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:4">
+      <x:c r="A1" s="0" t="s">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="B1" s="0" t="s">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="C1" s="0" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="D1" s="0" t="s">
+        <x:v>134</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:4">
+      <x:c r="A2" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:4">
+      <x:c r="A3" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>136</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:4">
+      <x:c r="A4" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="E11" s="0" t="s">
-        <x:v>125</x:v>
+      <x:c r="C4" s="0" t="s">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>137</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>